<commit_message>
chore: run 2026-05-31 16:26 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_31_05_2026.xlsx
+++ b/logs/Consolidado_31_05_2026.xlsx
@@ -790,7 +790,7 @@
         <v>424</v>
       </c>
       <c r="C9" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -29314,43 +29314,43 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>P&amp;C</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Protetor Solar Spray Adulto SPF50</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>https://www.perfumesecompanhia.pt/pt/avene-protetor-solar-spray-adulto-spf50/428120.html</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>70972M</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -35119,43 +35119,43 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="7" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="B160" s="7" t="inlineStr">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
         <is>
           <t>P&amp;C</t>
         </is>
       </c>
-      <c r="C160" s="7" t="inlineStr">
+      <c r="C160" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="D160" s="7" t="inlineStr">
+      <c r="D160" s="3" t="inlineStr">
         <is>
           <t>Dermalibour + Barrier - Creme Barreira</t>
         </is>
       </c>
-      <c r="E160" s="7" t="inlineStr">
+      <c r="E160" s="3" t="inlineStr">
         <is>
           <t>https://www.perfumesecompanhia.pt/pt/a-derma-dermalibour-barrier---creme-barreira/431665.html</t>
         </is>
       </c>
-      <c r="F160" s="7" t="inlineStr"/>
-      <c r="G160" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="H160" s="7" t="inlineStr">
+      <c r="F160" s="3" t="inlineStr"/>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="inlineStr">
         <is>
           <t>74518M</t>
         </is>
       </c>
-      <c r="I160" s="7" t="inlineStr">
+      <c r="I160" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -38129,43 +38129,43 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="7" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="B230" s="7" t="inlineStr">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
         <is>
           <t>P&amp;C</t>
         </is>
       </c>
-      <c r="C230" s="7" t="inlineStr">
+      <c r="C230" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="D230" s="7" t="inlineStr">
+      <c r="D230" s="3" t="inlineStr">
         <is>
           <t>Kertyol PSO Champô</t>
         </is>
       </c>
-      <c r="E230" s="7" t="inlineStr">
+      <c r="E230" s="3" t="inlineStr">
         <is>
           <t>https://www.perfumesecompanhia.pt/pt/ducray-kertyol-pso-champo/431572.html</t>
         </is>
       </c>
-      <c r="F230" s="7" t="inlineStr"/>
-      <c r="G230" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="H230" s="7" t="inlineStr">
+      <c r="F230" s="3" t="inlineStr"/>
+      <c r="G230" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr">
         <is>
           <t>74425M</t>
         </is>
       </c>
-      <c r="I230" s="7" t="inlineStr">
+      <c r="I230" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -40752,43 +40752,43 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="7" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="B291" s="7" t="inlineStr">
+      <c r="A291" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="B291" s="5" t="inlineStr">
         <is>
           <t>P&amp;C</t>
         </is>
       </c>
-      <c r="C291" s="7" t="inlineStr">
+      <c r="C291" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="D291" s="7" t="inlineStr">
+      <c r="D291" s="5" t="inlineStr">
         <is>
           <t>Champô Figo da Índia Hidratante Cabelo Baço</t>
         </is>
       </c>
-      <c r="E291" s="7" t="inlineStr">
+      <c r="E291" s="5" t="inlineStr">
         <is>
           <t>https://www.perfumesecompanhia.pt/pt/klorane-champo-figo-da-india-hidratante-cabelo-baco/428206.html</t>
         </is>
       </c>
-      <c r="F291" s="7" t="inlineStr"/>
-      <c r="G291" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="H291" s="7" t="inlineStr">
+      <c r="F291" s="5" t="inlineStr"/>
+      <c r="G291" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="H291" s="5" t="inlineStr">
         <is>
           <t>71059M</t>
         </is>
       </c>
-      <c r="I291" s="7" t="inlineStr">
+      <c r="I291" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -44536,43 +44536,43 @@
       </c>
     </row>
     <row r="379">
-      <c r="A379" s="7" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="B379" s="7" t="inlineStr">
+      <c r="A379" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="B379" s="5" t="inlineStr">
         <is>
           <t>P&amp;C</t>
         </is>
       </c>
-      <c r="C379" s="7" t="inlineStr">
+      <c r="C379" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="D379" s="7" t="inlineStr">
+      <c r="D379" s="5" t="inlineStr">
         <is>
           <t>Head Spa Complexe 5 Concentrado Vegetal Estimulante</t>
         </is>
       </c>
-      <c r="E379" s="7" t="inlineStr">
+      <c r="E379" s="5" t="inlineStr">
         <is>
           <t>https://www.perfumesecompanhia.pt/pt/rene-furterer-head-spa-complexe-5-concentrado-vegetal-estimulante/428128.html</t>
         </is>
       </c>
-      <c r="F379" s="7" t="inlineStr"/>
-      <c r="G379" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="H379" s="7" t="inlineStr">
+      <c r="F379" s="5" t="inlineStr"/>
+      <c r="G379" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="H379" s="5" t="inlineStr">
         <is>
           <t>70980M</t>
         </is>
       </c>
-      <c r="I379" s="7" t="inlineStr">
+      <c r="I379" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-05-31 20:03 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_31_05_2026.xlsx
+++ b/logs/Consolidado_31_05_2026.xlsx
@@ -752,10 +752,10 @@
         <v>102</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -18656,11 +18656,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>6490926</t>
-        </is>
-      </c>
+      <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr">
         <is>
           <t>28%</t>
@@ -26313,40 +26309,40 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>Elgydium
 Gel Dentes Sensíveis
 75 ml</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="D67" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/gel-dentes-sensiveis-3000688.html</t>
         </is>
       </c>
-      <c r="E67" s="5" t="inlineStr"/>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr"/>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
         <is>
           <t>3000688</t>
         </is>
       </c>
-      <c r="H67" s="5" t="inlineStr">
+      <c r="H67" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -28358,7 +28354,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>81060M</t>
+          <t>438077</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -28401,7 +28397,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>77678M</t>
+          <t>428292</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -28444,7 +28440,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>76498M</t>
+          <t>433636</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -28487,7 +28483,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>76687M</t>
+          <t>433825</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -28530,7 +28526,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>70827M</t>
+          <t>427975</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -28573,7 +28569,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>74575M</t>
+          <t>431722</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -28616,7 +28612,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>70829M</t>
+          <t>427977</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -28659,7 +28655,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>71165M</t>
+          <t>428313</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -28702,7 +28698,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>70812M</t>
+          <t>427960</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -28745,7 +28741,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>76497M</t>
+          <t>433635</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -28788,7 +28784,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>77685M</t>
+          <t>427936</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -28831,7 +28827,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>77677M</t>
+          <t>428309</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -28874,7 +28870,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>76495M</t>
+          <t>433633</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -28917,7 +28913,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>70963M</t>
+          <t>428111</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -28960,7 +28956,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>71167M</t>
+          <t>428315</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -29003,7 +28999,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>70826M</t>
+          <t>427974</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -29046,7 +29042,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>81062M</t>
+          <t>438079</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -29089,7 +29085,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>70959M</t>
+          <t>428107</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -29132,7 +29128,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>78158M</t>
+          <t>435214</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -29175,7 +29171,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>70830M</t>
+          <t>427978</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -29218,7 +29214,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>76686M</t>
+          <t>433824</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -29261,7 +29257,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>70809M</t>
+          <t>427957</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -29304,7 +29300,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>71171M</t>
+          <t>428319</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -29347,7 +29343,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>70972M</t>
+          <t>428120</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -29390,7 +29386,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>77681M</t>
+          <t>428109</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -29433,7 +29429,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>71177M</t>
+          <t>428325</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -29476,7 +29472,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>77680M</t>
+          <t>428123</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -29519,7 +29515,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>70951M</t>
+          <t>428099</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -29562,7 +29558,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>71155M</t>
+          <t>428303</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -29605,7 +29601,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>70962M</t>
+          <t>428110</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -29648,7 +29644,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>70956M</t>
+          <t>428104</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -29691,7 +29687,7 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>74582M</t>
+          <t>431729</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -29734,7 +29730,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>70810M</t>
+          <t>427958</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -29777,7 +29773,7 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>71157M</t>
+          <t>428305</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -29820,7 +29816,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>70834M</t>
+          <t>427982</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -29863,7 +29859,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>70832M</t>
+          <t>427980</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -29906,7 +29902,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>81061M</t>
+          <t>438078</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -29949,7 +29945,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>70818M</t>
+          <t>427966</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -29992,7 +29988,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>70817M</t>
+          <t>427965</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -30035,7 +30031,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>71149M</t>
+          <t>428297</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -30078,7 +30074,7 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>70833M</t>
+          <t>427981</t>
         </is>
       </c>
       <c r="I42" s="7" t="inlineStr">
@@ -30121,7 +30117,7 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>70953M</t>
+          <t>428101</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -30164,7 +30160,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>70955M</t>
+          <t>428102</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -30207,7 +30203,7 @@
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>70969M</t>
+          <t>428117</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -30250,7 +30246,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>81065M</t>
+          <t>438082</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -30293,7 +30289,7 @@
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>70823M</t>
+          <t>427971</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
@@ -30336,7 +30332,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>88062M</t>
+          <t>445067</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -30379,7 +30375,7 @@
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>70814M</t>
+          <t>427962</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
@@ -30422,7 +30418,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>70843M</t>
+          <t>427991</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -30465,7 +30461,7 @@
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>71147M</t>
+          <t>428295</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
@@ -30508,7 +30504,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>70801M</t>
+          <t>427949</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -30551,7 +30547,7 @@
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>71148M</t>
+          <t>428296</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
@@ -30594,7 +30590,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>76496M</t>
+          <t>433634</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -30637,7 +30633,7 @@
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>74579M</t>
+          <t>431726</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -30680,7 +30676,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>74584M</t>
+          <t>431731</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -30723,7 +30719,7 @@
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>74574M</t>
+          <t>431721</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
@@ -30766,7 +30762,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>70964M</t>
+          <t>428112</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -30809,7 +30805,7 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>71175M</t>
+          <t>428323</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
@@ -30852,7 +30848,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>70842M</t>
+          <t>427990</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -30895,7 +30891,7 @@
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>77682M</t>
+          <t>427988</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
@@ -30938,7 +30934,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>70966M</t>
+          <t>428114</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -30981,7 +30977,7 @@
       </c>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>79052M</t>
+          <t>436085</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
@@ -31024,7 +31020,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>70811M</t>
+          <t>427959</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -31067,7 +31063,7 @@
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>70835M</t>
+          <t>427983</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
@@ -31110,7 +31106,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>70798M</t>
+          <t>427946</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -31153,7 +31149,7 @@
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>70844M</t>
+          <t>427992</t>
         </is>
       </c>
       <c r="I67" s="5" t="inlineStr">
@@ -31196,7 +31192,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>74588M</t>
+          <t>431735</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -31239,7 +31235,7 @@
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>70799M</t>
+          <t>427947</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
@@ -31282,7 +31278,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>70965M</t>
+          <t>428113</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -31325,7 +31321,7 @@
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>70808M</t>
+          <t>427956</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
@@ -31368,7 +31364,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>70820M</t>
+          <t>427968</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -31411,7 +31407,7 @@
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>70836M</t>
+          <t>427984</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
@@ -31454,7 +31450,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>70974M</t>
+          <t>428122</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -31497,7 +31493,7 @@
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>70949M</t>
+          <t>428097</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
@@ -31540,7 +31536,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>70791M</t>
+          <t>427939</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -31583,7 +31579,7 @@
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>70979M</t>
+          <t>428127</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
@@ -31626,7 +31622,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>74580M</t>
+          <t>431727</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -31669,7 +31665,7 @@
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>71159M</t>
+          <t>428307</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
@@ -31712,7 +31708,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>77594M</t>
+          <t>431723</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -31755,7 +31751,7 @@
       </c>
       <c r="H81" s="5" t="inlineStr">
         <is>
-          <t>74581M</t>
+          <t>431728</t>
         </is>
       </c>
       <c r="I81" s="5" t="inlineStr">
@@ -31798,7 +31794,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>74587M</t>
+          <t>431734</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
@@ -31841,7 +31837,7 @@
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>70828M</t>
+          <t>427976</t>
         </is>
       </c>
       <c r="I83" s="7" t="inlineStr">
@@ -31884,7 +31880,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>71153M</t>
+          <t>428301</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -31927,7 +31923,7 @@
       </c>
       <c r="H85" s="5" t="inlineStr">
         <is>
-          <t>70794M</t>
+          <t>427942</t>
         </is>
       </c>
       <c r="I85" s="5" t="inlineStr">
@@ -31970,7 +31966,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>70804M</t>
+          <t>427952</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -32013,7 +32009,7 @@
       </c>
       <c r="H87" s="5" t="inlineStr">
         <is>
-          <t>71169M</t>
+          <t>428317</t>
         </is>
       </c>
       <c r="I87" s="5" t="inlineStr">
@@ -32056,7 +32052,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>70950M</t>
+          <t>428098</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -32099,7 +32095,7 @@
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>70952M</t>
+          <t>428100</t>
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
@@ -32142,7 +32138,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>74578M</t>
+          <t>431725</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -32185,7 +32181,7 @@
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>71173M</t>
+          <t>428321</t>
         </is>
       </c>
       <c r="I91" s="5" t="inlineStr">
@@ -32228,7 +32224,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>70803M</t>
+          <t>427951</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -32271,7 +32267,7 @@
       </c>
       <c r="H93" s="5" t="inlineStr">
         <is>
-          <t>70792M</t>
+          <t>427940</t>
         </is>
       </c>
       <c r="I93" s="5" t="inlineStr">
@@ -32314,7 +32310,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>81063M</t>
+          <t>438080</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -32357,7 +32353,7 @@
       </c>
       <c r="H95" s="5" t="inlineStr">
         <is>
-          <t>70946M</t>
+          <t>428094</t>
         </is>
       </c>
       <c r="I95" s="5" t="inlineStr">
@@ -32400,7 +32396,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>70948M</t>
+          <t>428096</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -32443,7 +32439,7 @@
       </c>
       <c r="H97" s="5" t="inlineStr">
         <is>
-          <t>77911M</t>
+          <t>434993</t>
         </is>
       </c>
       <c r="I97" s="5" t="inlineStr">
@@ -32486,7 +32482,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>70816M</t>
+          <t>427964</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
@@ -32529,7 +32525,7 @@
       </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t>70958M</t>
+          <t>428106</t>
         </is>
       </c>
       <c r="I99" s="5" t="inlineStr">
@@ -32572,7 +32568,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>71146M</t>
+          <t>428294</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -32615,7 +32611,7 @@
       </c>
       <c r="H101" s="5" t="inlineStr">
         <is>
-          <t>70824M</t>
+          <t>427972</t>
         </is>
       </c>
       <c r="I101" s="5" t="inlineStr">
@@ -32658,7 +32654,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>71151M</t>
+          <t>428299</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -32701,7 +32697,7 @@
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>70957M</t>
+          <t>428105</t>
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr">
@@ -32744,7 +32740,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>70831M</t>
+          <t>427979</t>
         </is>
       </c>
       <c r="I104" s="3" t="inlineStr">
@@ -32787,7 +32783,7 @@
       </c>
       <c r="H105" s="5" t="inlineStr">
         <is>
-          <t>70802M</t>
+          <t>427950</t>
         </is>
       </c>
       <c r="I105" s="5" t="inlineStr">
@@ -32830,7 +32826,7 @@
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>70821M</t>
+          <t>427969</t>
         </is>
       </c>
       <c r="I106" s="3" t="inlineStr">
@@ -32873,7 +32869,7 @@
       </c>
       <c r="H107" s="5" t="inlineStr">
         <is>
-          <t>70819M</t>
+          <t>427967</t>
         </is>
       </c>
       <c r="I107" s="5" t="inlineStr">
@@ -32916,7 +32912,7 @@
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>70968M</t>
+          <t>428116</t>
         </is>
       </c>
       <c r="I108" s="3" t="inlineStr">
@@ -32959,7 +32955,7 @@
       </c>
       <c r="H109" s="5" t="inlineStr">
         <is>
-          <t>70822M</t>
+          <t>427970</t>
         </is>
       </c>
       <c r="I109" s="5" t="inlineStr">
@@ -33002,7 +32998,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>77684M</t>
+          <t>427944</t>
         </is>
       </c>
       <c r="I110" s="3" t="inlineStr">
@@ -33045,7 +33041,7 @@
       </c>
       <c r="H111" s="5" t="inlineStr">
         <is>
-          <t>70971M</t>
+          <t>428119</t>
         </is>
       </c>
       <c r="I111" s="5" t="inlineStr">
@@ -33088,7 +33084,7 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>70954M</t>
+          <t>428103</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -33131,7 +33127,7 @@
       </c>
       <c r="H113" s="5" t="inlineStr">
         <is>
-          <t>70967M</t>
+          <t>428115</t>
         </is>
       </c>
       <c r="I113" s="5" t="inlineStr">
@@ -33174,7 +33170,7 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>70797M</t>
+          <t>427945</t>
         </is>
       </c>
       <c r="I114" s="3" t="inlineStr">
@@ -33217,7 +33213,7 @@
       </c>
       <c r="H115" s="5" t="inlineStr">
         <is>
-          <t>74586M</t>
+          <t>431733</t>
         </is>
       </c>
       <c r="I115" s="5" t="inlineStr">
@@ -33260,7 +33256,7 @@
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>80972M</t>
+          <t>437988</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -33303,7 +33299,7 @@
       </c>
       <c r="H117" s="5" t="inlineStr">
         <is>
-          <t>70807M</t>
+          <t>427955</t>
         </is>
       </c>
       <c r="I117" s="5" t="inlineStr">
@@ -33346,7 +33342,7 @@
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>70838M</t>
+          <t>427986</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -33389,7 +33385,7 @@
       </c>
       <c r="H119" s="5" t="inlineStr">
         <is>
-          <t>70806M</t>
+          <t>427954</t>
         </is>
       </c>
       <c r="I119" s="5" t="inlineStr">
@@ -33432,7 +33428,7 @@
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>88061M</t>
+          <t>445066</t>
         </is>
       </c>
       <c r="I120" s="3" t="inlineStr">
@@ -33475,7 +33471,7 @@
       </c>
       <c r="H121" s="5" t="inlineStr">
         <is>
-          <t>83058M</t>
+          <t>440070</t>
         </is>
       </c>
       <c r="I121" s="5" t="inlineStr">
@@ -33518,7 +33514,7 @@
       </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
-          <t>81059M</t>
+          <t>438076</t>
         </is>
       </c>
       <c r="I122" s="3" t="inlineStr">
@@ -33561,7 +33557,7 @@
       </c>
       <c r="H123" s="5" t="inlineStr">
         <is>
-          <t>70947M</t>
+          <t>428095</t>
         </is>
       </c>
       <c r="I123" s="5" t="inlineStr">
@@ -33604,7 +33600,7 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>70837M</t>
+          <t>427985</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -33647,7 +33643,7 @@
       </c>
       <c r="H125" s="5" t="inlineStr">
         <is>
-          <t>80974M</t>
+          <t>437990</t>
         </is>
       </c>
       <c r="I125" s="5" t="inlineStr">
@@ -33690,7 +33686,7 @@
       </c>
       <c r="H126" s="7" t="inlineStr">
         <is>
-          <t>70795M</t>
+          <t>427943</t>
         </is>
       </c>
       <c r="I126" s="7" t="inlineStr">
@@ -33733,7 +33729,7 @@
       </c>
       <c r="H127" s="5" t="inlineStr">
         <is>
-          <t>87425M</t>
+          <t>444431</t>
         </is>
       </c>
       <c r="I127" s="5" t="inlineStr">
@@ -33776,7 +33772,7 @@
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>80776M</t>
+          <t>437793</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -33819,7 +33815,7 @@
       </c>
       <c r="H129" s="5" t="inlineStr">
         <is>
-          <t>70973M</t>
+          <t>428121</t>
         </is>
       </c>
       <c r="I129" s="5" t="inlineStr">
@@ -33862,7 +33858,7 @@
       </c>
       <c r="H130" s="3" t="inlineStr">
         <is>
-          <t>70815M</t>
+          <t>427963</t>
         </is>
       </c>
       <c r="I130" s="3" t="inlineStr">
@@ -33905,7 +33901,7 @@
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
-          <t>80774M</t>
+          <t>437791</t>
         </is>
       </c>
       <c r="I131" s="5" t="inlineStr">
@@ -33948,7 +33944,7 @@
       </c>
       <c r="H132" s="3" t="inlineStr">
         <is>
-          <t>70825M</t>
+          <t>427973</t>
         </is>
       </c>
       <c r="I132" s="3" t="inlineStr">
@@ -33991,7 +33987,7 @@
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
-          <t>70841M</t>
+          <t>427989</t>
         </is>
       </c>
       <c r="I133" s="5" t="inlineStr">
@@ -34034,7 +34030,7 @@
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>79051M</t>
+          <t>436084</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -34077,7 +34073,7 @@
       </c>
       <c r="H135" s="5" t="inlineStr">
         <is>
-          <t>70805M</t>
+          <t>427953</t>
         </is>
       </c>
       <c r="I135" s="5" t="inlineStr">
@@ -34120,7 +34116,7 @@
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>70813M</t>
+          <t>427961</t>
         </is>
       </c>
       <c r="I136" s="7" t="inlineStr">
@@ -34163,7 +34159,7 @@
       </c>
       <c r="H137" s="5" t="inlineStr">
         <is>
-          <t>74572M</t>
+          <t>431719</t>
         </is>
       </c>
       <c r="I137" s="5" t="inlineStr">
@@ -34206,7 +34202,7 @@
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
-          <t>74503M</t>
+          <t>431649</t>
         </is>
       </c>
       <c r="I138" s="3" t="inlineStr">
@@ -34249,7 +34245,7 @@
       </c>
       <c r="H139" s="5" t="inlineStr">
         <is>
-          <t>74540M</t>
+          <t>431687</t>
         </is>
       </c>
       <c r="I139" s="5" t="inlineStr">
@@ -34292,7 +34288,7 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>76685M</t>
+          <t>433823</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -34335,7 +34331,7 @@
       </c>
       <c r="H141" s="5" t="inlineStr">
         <is>
-          <t>88657M</t>
+          <t>431637</t>
         </is>
       </c>
       <c r="I141" s="5" t="inlineStr">
@@ -34378,7 +34374,7 @@
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>74495M</t>
+          <t>431642</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -34421,7 +34417,7 @@
       </c>
       <c r="H143" s="5" t="inlineStr">
         <is>
-          <t>74515M</t>
+          <t>431663</t>
         </is>
       </c>
       <c r="I143" s="5" t="inlineStr">
@@ -34464,7 +34460,7 @@
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>74500M</t>
+          <t>431647</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -34507,7 +34503,7 @@
       </c>
       <c r="H145" s="5" t="inlineStr">
         <is>
-          <t>74513M</t>
+          <t>431660</t>
         </is>
       </c>
       <c r="I145" s="5" t="inlineStr">
@@ -34550,7 +34546,7 @@
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>74573M</t>
+          <t>431720</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -34593,7 +34589,7 @@
       </c>
       <c r="H147" s="5" t="inlineStr">
         <is>
-          <t>74545M</t>
+          <t>431692</t>
         </is>
       </c>
       <c r="I147" s="5" t="inlineStr">
@@ -34636,7 +34632,7 @@
       </c>
       <c r="H148" s="7" t="inlineStr">
         <is>
-          <t>74532M</t>
+          <t>431679</t>
         </is>
       </c>
       <c r="I148" s="7" t="inlineStr">
@@ -34679,7 +34675,7 @@
       </c>
       <c r="H149" s="7" t="inlineStr">
         <is>
-          <t>74531M</t>
+          <t>431678</t>
         </is>
       </c>
       <c r="I149" s="7" t="inlineStr">
@@ -34722,7 +34718,7 @@
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>74496M</t>
+          <t>431643</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
@@ -34765,7 +34761,7 @@
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
-          <t>74498M</t>
+          <t>431645</t>
         </is>
       </c>
       <c r="I151" s="5" t="inlineStr">
@@ -34808,7 +34804,7 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>74558M</t>
+          <t>431705</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
@@ -34851,7 +34847,7 @@
       </c>
       <c r="H153" s="5" t="inlineStr">
         <is>
-          <t>74520M</t>
+          <t>431667</t>
         </is>
       </c>
       <c r="I153" s="5" t="inlineStr">
@@ -34894,7 +34890,7 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>74512M</t>
+          <t>431659</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -34937,7 +34933,7 @@
       </c>
       <c r="H155" s="5" t="inlineStr">
         <is>
-          <t>74505M</t>
+          <t>431652</t>
         </is>
       </c>
       <c r="I155" s="5" t="inlineStr">
@@ -34980,7 +34976,7 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
-          <t>74560M</t>
+          <t>431707</t>
         </is>
       </c>
       <c r="I156" s="3" t="inlineStr">
@@ -35023,7 +35019,7 @@
       </c>
       <c r="H157" s="5" t="inlineStr">
         <is>
-          <t>74517M</t>
+          <t>431664</t>
         </is>
       </c>
       <c r="I157" s="5" t="inlineStr">
@@ -35066,7 +35062,7 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>74562M</t>
+          <t>431709</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
@@ -35109,7 +35105,7 @@
       </c>
       <c r="H159" s="5" t="inlineStr">
         <is>
-          <t>74570M</t>
+          <t>431717</t>
         </is>
       </c>
       <c r="I159" s="5" t="inlineStr">
@@ -35152,7 +35148,7 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
-          <t>74518M</t>
+          <t>431665</t>
         </is>
       </c>
       <c r="I160" s="3" t="inlineStr">
@@ -35195,7 +35191,7 @@
       </c>
       <c r="H161" s="7" t="inlineStr">
         <is>
-          <t>74533M</t>
+          <t>431680</t>
         </is>
       </c>
       <c r="I161" s="7" t="inlineStr">
@@ -35238,7 +35234,7 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>74557M</t>
+          <t>431704</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -35281,7 +35277,7 @@
       </c>
       <c r="H163" s="5" t="inlineStr">
         <is>
-          <t>74547M</t>
+          <t>431694</t>
         </is>
       </c>
       <c r="I163" s="5" t="inlineStr">
@@ -35324,7 +35320,7 @@
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>74550M</t>
+          <t>431697</t>
         </is>
       </c>
       <c r="I164" s="3" t="inlineStr">
@@ -35367,7 +35363,7 @@
       </c>
       <c r="H165" s="5" t="inlineStr">
         <is>
-          <t>74566M</t>
+          <t>431713</t>
         </is>
       </c>
       <c r="I165" s="5" t="inlineStr">
@@ -35410,7 +35406,7 @@
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>74563M</t>
+          <t>431710</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
@@ -35453,7 +35449,7 @@
       </c>
       <c r="H167" s="5" t="inlineStr">
         <is>
-          <t>74565M</t>
+          <t>431712</t>
         </is>
       </c>
       <c r="I167" s="5" t="inlineStr">
@@ -35496,7 +35492,7 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>74541M</t>
+          <t>431688</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -35539,7 +35535,7 @@
       </c>
       <c r="H169" s="5" t="inlineStr">
         <is>
-          <t>77416M</t>
+          <t>434552</t>
         </is>
       </c>
       <c r="I169" s="5" t="inlineStr">
@@ -35582,7 +35578,7 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>74526M</t>
+          <t>431673</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -35625,7 +35621,7 @@
       </c>
       <c r="H171" s="5" t="inlineStr">
         <is>
-          <t>74492M</t>
+          <t>431639</t>
         </is>
       </c>
       <c r="I171" s="5" t="inlineStr">
@@ -35668,7 +35664,7 @@
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>77417M</t>
+          <t>434553</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -35711,7 +35707,7 @@
       </c>
       <c r="H173" s="5" t="inlineStr">
         <is>
-          <t>74494M</t>
+          <t>431641</t>
         </is>
       </c>
       <c r="I173" s="5" t="inlineStr">
@@ -35754,7 +35750,7 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>77415M</t>
+          <t>434551</t>
         </is>
       </c>
       <c r="I174" s="3" t="inlineStr">
@@ -35797,7 +35793,7 @@
       </c>
       <c r="H175" s="5" t="inlineStr">
         <is>
-          <t>74539M</t>
+          <t>431686</t>
         </is>
       </c>
       <c r="I175" s="5" t="inlineStr">
@@ -35840,7 +35836,7 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>74525M</t>
+          <t>431672</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -35883,7 +35879,7 @@
       </c>
       <c r="H177" s="5" t="inlineStr">
         <is>
-          <t>74564M</t>
+          <t>431711</t>
         </is>
       </c>
       <c r="I177" s="5" t="inlineStr">
@@ -35926,7 +35922,7 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>74568M</t>
+          <t>431715</t>
         </is>
       </c>
       <c r="I178" s="3" t="inlineStr">
@@ -35969,7 +35965,7 @@
       </c>
       <c r="H179" s="5" t="inlineStr">
         <is>
-          <t>74569M</t>
+          <t>431716</t>
         </is>
       </c>
       <c r="I179" s="5" t="inlineStr">
@@ -36012,7 +36008,7 @@
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>74534M</t>
+          <t>431681</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -36055,7 +36051,7 @@
       </c>
       <c r="H181" s="5" t="inlineStr">
         <is>
-          <t>74552M</t>
+          <t>431699</t>
         </is>
       </c>
       <c r="I181" s="5" t="inlineStr">
@@ -36098,7 +36094,7 @@
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>74522M</t>
+          <t>431670</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
@@ -36141,7 +36137,7 @@
       </c>
       <c r="H183" s="5" t="inlineStr">
         <is>
-          <t>74548M</t>
+          <t>431696</t>
         </is>
       </c>
       <c r="I183" s="5" t="inlineStr">
@@ -36184,7 +36180,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>74554M</t>
+          <t>431701</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
@@ -36227,7 +36223,7 @@
       </c>
       <c r="H185" s="5" t="inlineStr">
         <is>
-          <t>74538M</t>
+          <t>431685</t>
         </is>
       </c>
       <c r="I185" s="5" t="inlineStr">
@@ -36270,7 +36266,7 @@
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>74528M</t>
+          <t>431675</t>
         </is>
       </c>
       <c r="I186" s="3" t="inlineStr">
@@ -36313,7 +36309,7 @@
       </c>
       <c r="H187" s="5" t="inlineStr">
         <is>
-          <t>74551M</t>
+          <t>431698</t>
         </is>
       </c>
       <c r="I187" s="5" t="inlineStr">
@@ -36356,7 +36352,7 @@
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>74555M</t>
+          <t>431702</t>
         </is>
       </c>
       <c r="I188" s="3" t="inlineStr">
@@ -36399,7 +36395,7 @@
       </c>
       <c r="H189" s="5" t="inlineStr">
         <is>
-          <t>88044M</t>
+          <t>445049</t>
         </is>
       </c>
       <c r="I189" s="5" t="inlineStr">
@@ -36442,7 +36438,7 @@
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>74529M</t>
+          <t>431676</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
@@ -36485,7 +36481,7 @@
       </c>
       <c r="H191" s="5" t="inlineStr">
         <is>
-          <t>74489M</t>
+          <t>431636</t>
         </is>
       </c>
       <c r="I191" s="5" t="inlineStr">
@@ -36528,7 +36524,7 @@
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>74511M</t>
+          <t>431658</t>
         </is>
       </c>
       <c r="I192" s="3" t="inlineStr">
@@ -36571,7 +36567,7 @@
       </c>
       <c r="H193" s="5" t="inlineStr">
         <is>
-          <t>74530M</t>
+          <t>431677</t>
         </is>
       </c>
       <c r="I193" s="5" t="inlineStr">
@@ -36614,7 +36610,7 @@
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>74507M</t>
+          <t>431654</t>
         </is>
       </c>
       <c r="I194" s="3" t="inlineStr">
@@ -36657,7 +36653,7 @@
       </c>
       <c r="H195" s="5" t="inlineStr">
         <is>
-          <t>88041M</t>
+          <t>445046</t>
         </is>
       </c>
       <c r="I195" s="5" t="inlineStr">
@@ -36700,7 +36696,7 @@
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>88042M</t>
+          <t>445047</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -36743,7 +36739,7 @@
       </c>
       <c r="H197" s="5" t="inlineStr">
         <is>
-          <t>74542M</t>
+          <t>431689</t>
         </is>
       </c>
       <c r="I197" s="5" t="inlineStr">
@@ -36786,7 +36782,7 @@
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>88043M</t>
+          <t>445048</t>
         </is>
       </c>
       <c r="I198" s="3" t="inlineStr">
@@ -36829,7 +36825,7 @@
       </c>
       <c r="H199" s="5" t="inlineStr">
         <is>
-          <t>74571M</t>
+          <t>431718</t>
         </is>
       </c>
       <c r="I199" s="5" t="inlineStr">
@@ -36872,7 +36868,7 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>74536M</t>
+          <t>431683</t>
         </is>
       </c>
       <c r="I200" s="3" t="inlineStr">
@@ -36915,7 +36911,7 @@
       </c>
       <c r="H201" s="5" t="inlineStr">
         <is>
-          <t>74509M</t>
+          <t>431656</t>
         </is>
       </c>
       <c r="I201" s="5" t="inlineStr">
@@ -36958,7 +36954,7 @@
       </c>
       <c r="H202" s="3" t="inlineStr">
         <is>
-          <t>87916M</t>
+          <t>444921</t>
         </is>
       </c>
       <c r="I202" s="3" t="inlineStr">
@@ -37001,7 +36997,7 @@
       </c>
       <c r="H203" s="5" t="inlineStr">
         <is>
-          <t>74521M</t>
+          <t>431668</t>
         </is>
       </c>
       <c r="I203" s="5" t="inlineStr">
@@ -37044,7 +37040,7 @@
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>74561M</t>
+          <t>431708</t>
         </is>
       </c>
       <c r="I204" s="3" t="inlineStr">
@@ -37087,7 +37083,7 @@
       </c>
       <c r="H205" s="5" t="inlineStr">
         <is>
-          <t>74567M</t>
+          <t>431714</t>
         </is>
       </c>
       <c r="I205" s="5" t="inlineStr">
@@ -37130,7 +37126,7 @@
       </c>
       <c r="H206" s="3" t="inlineStr">
         <is>
-          <t>74537M</t>
+          <t>431684</t>
         </is>
       </c>
       <c r="I206" s="3" t="inlineStr">
@@ -37173,7 +37169,7 @@
       </c>
       <c r="H207" s="5" t="inlineStr">
         <is>
-          <t>74453M</t>
+          <t>431601</t>
         </is>
       </c>
       <c r="I207" s="5" t="inlineStr">
@@ -37216,7 +37212,7 @@
       </c>
       <c r="H208" s="3" t="inlineStr">
         <is>
-          <t>74414M</t>
+          <t>431561</t>
         </is>
       </c>
       <c r="I208" s="3" t="inlineStr">
@@ -37259,7 +37255,7 @@
       </c>
       <c r="H209" s="7" t="inlineStr">
         <is>
-          <t>74464M</t>
+          <t>431611</t>
         </is>
       </c>
       <c r="I209" s="7" t="inlineStr">
@@ -37302,7 +37298,7 @@
       </c>
       <c r="H210" s="3" t="inlineStr">
         <is>
-          <t>74484M</t>
+          <t>431631</t>
         </is>
       </c>
       <c r="I210" s="3" t="inlineStr">
@@ -37345,7 +37341,7 @@
       </c>
       <c r="H211" s="5" t="inlineStr">
         <is>
-          <t>74431M</t>
+          <t>431577</t>
         </is>
       </c>
       <c r="I211" s="5" t="inlineStr">
@@ -37388,7 +37384,7 @@
       </c>
       <c r="H212" s="3" t="inlineStr">
         <is>
-          <t>74463M</t>
+          <t>431610</t>
         </is>
       </c>
       <c r="I212" s="3" t="inlineStr">
@@ -37431,7 +37427,7 @@
       </c>
       <c r="H213" s="7" t="inlineStr">
         <is>
-          <t>74424M</t>
+          <t>431571</t>
         </is>
       </c>
       <c r="I213" s="7" t="inlineStr">
@@ -37474,7 +37470,7 @@
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>74416M</t>
+          <t>431563</t>
         </is>
       </c>
       <c r="I214" s="3" t="inlineStr">
@@ -37517,7 +37513,7 @@
       </c>
       <c r="H215" s="5" t="inlineStr">
         <is>
-          <t>74482M</t>
+          <t>431629</t>
         </is>
       </c>
       <c r="I215" s="5" t="inlineStr">
@@ -37560,7 +37556,7 @@
       </c>
       <c r="H216" s="3" t="inlineStr">
         <is>
-          <t>74423M</t>
+          <t>431569</t>
         </is>
       </c>
       <c r="I216" s="3" t="inlineStr">
@@ -37603,7 +37599,7 @@
       </c>
       <c r="H217" s="5" t="inlineStr">
         <is>
-          <t>74436M</t>
+          <t>431582</t>
         </is>
       </c>
       <c r="I217" s="5" t="inlineStr">
@@ -37646,7 +37642,7 @@
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
-          <t>74446M</t>
+          <t>431593</t>
         </is>
       </c>
       <c r="I218" s="3" t="inlineStr">
@@ -37689,7 +37685,7 @@
       </c>
       <c r="H219" s="5" t="inlineStr">
         <is>
-          <t>74473M</t>
+          <t>431620</t>
         </is>
       </c>
       <c r="I219" s="5" t="inlineStr">
@@ -37732,7 +37728,7 @@
       </c>
       <c r="H220" s="3" t="inlineStr">
         <is>
-          <t>74415M</t>
+          <t>431562</t>
         </is>
       </c>
       <c r="I220" s="3" t="inlineStr">
@@ -37775,7 +37771,7 @@
       </c>
       <c r="H221" s="5" t="inlineStr">
         <is>
-          <t>74449M</t>
+          <t>431595</t>
         </is>
       </c>
       <c r="I221" s="5" t="inlineStr">
@@ -37818,7 +37814,7 @@
       </c>
       <c r="H222" s="3" t="inlineStr">
         <is>
-          <t>74451M</t>
+          <t>431597</t>
         </is>
       </c>
       <c r="I222" s="3" t="inlineStr">
@@ -37861,7 +37857,7 @@
       </c>
       <c r="H223" s="5" t="inlineStr">
         <is>
-          <t>74419M</t>
+          <t>431566</t>
         </is>
       </c>
       <c r="I223" s="5" t="inlineStr">
@@ -37904,7 +37900,7 @@
       </c>
       <c r="H224" s="3" t="inlineStr">
         <is>
-          <t>74434M</t>
+          <t>431579</t>
         </is>
       </c>
       <c r="I224" s="3" t="inlineStr">
@@ -37947,7 +37943,7 @@
       </c>
       <c r="H225" s="5" t="inlineStr">
         <is>
-          <t>74468M</t>
+          <t>431615</t>
         </is>
       </c>
       <c r="I225" s="5" t="inlineStr">
@@ -37990,7 +37986,7 @@
       </c>
       <c r="H226" s="3" t="inlineStr">
         <is>
-          <t>74488M</t>
+          <t>431635</t>
         </is>
       </c>
       <c r="I226" s="3" t="inlineStr">
@@ -38033,7 +38029,7 @@
       </c>
       <c r="H227" s="5" t="inlineStr">
         <is>
-          <t>74421M</t>
+          <t>431567</t>
         </is>
       </c>
       <c r="I227" s="5" t="inlineStr">
@@ -38076,7 +38072,7 @@
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>74455M</t>
+          <t>431602</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -38119,7 +38115,7 @@
       </c>
       <c r="H229" s="5" t="inlineStr">
         <is>
-          <t>74442M</t>
+          <t>431589</t>
         </is>
       </c>
       <c r="I229" s="5" t="inlineStr">
@@ -38162,7 +38158,7 @@
       </c>
       <c r="H230" s="3" t="inlineStr">
         <is>
-          <t>74425M</t>
+          <t>431572</t>
         </is>
       </c>
       <c r="I230" s="3" t="inlineStr">
@@ -38205,7 +38201,7 @@
       </c>
       <c r="H231" s="5" t="inlineStr">
         <is>
-          <t>74452M</t>
+          <t>431599</t>
         </is>
       </c>
       <c r="I231" s="5" t="inlineStr">
@@ -38248,7 +38244,7 @@
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>74474M</t>
+          <t>431621</t>
         </is>
       </c>
       <c r="I232" s="3" t="inlineStr">
@@ -38291,7 +38287,7 @@
       </c>
       <c r="H233" s="5" t="inlineStr">
         <is>
-          <t>80611M</t>
+          <t>437628</t>
         </is>
       </c>
       <c r="I233" s="5" t="inlineStr">
@@ -38334,7 +38330,7 @@
       </c>
       <c r="H234" s="3" t="inlineStr">
         <is>
-          <t>74426M</t>
+          <t>431573</t>
         </is>
       </c>
       <c r="I234" s="3" t="inlineStr">
@@ -38377,7 +38373,7 @@
       </c>
       <c r="H235" s="5" t="inlineStr">
         <is>
-          <t>74458M</t>
+          <t>431604</t>
         </is>
       </c>
       <c r="I235" s="5" t="inlineStr">
@@ -38420,7 +38416,7 @@
       </c>
       <c r="H236" s="3" t="inlineStr">
         <is>
-          <t>74465M</t>
+          <t>431612</t>
         </is>
       </c>
       <c r="I236" s="3" t="inlineStr">
@@ -38463,7 +38459,7 @@
       </c>
       <c r="H237" s="5" t="inlineStr">
         <is>
-          <t>74479M</t>
+          <t>431626</t>
         </is>
       </c>
       <c r="I237" s="5" t="inlineStr">
@@ -38506,7 +38502,7 @@
       </c>
       <c r="H238" s="3" t="inlineStr">
         <is>
-          <t>74485M</t>
+          <t>431632</t>
         </is>
       </c>
       <c r="I238" s="3" t="inlineStr">
@@ -38549,7 +38545,7 @@
       </c>
       <c r="H239" s="5" t="inlineStr">
         <is>
-          <t>74487M</t>
+          <t>431634</t>
         </is>
       </c>
       <c r="I239" s="5" t="inlineStr">
@@ -38592,7 +38588,7 @@
       </c>
       <c r="H240" s="3" t="inlineStr">
         <is>
-          <t>74441M</t>
+          <t>431588</t>
         </is>
       </c>
       <c r="I240" s="3" t="inlineStr">
@@ -38635,7 +38631,7 @@
       </c>
       <c r="H241" s="5" t="inlineStr">
         <is>
-          <t>74471M</t>
+          <t>431618</t>
         </is>
       </c>
       <c r="I241" s="5" t="inlineStr">
@@ -38678,7 +38674,7 @@
       </c>
       <c r="H242" s="3" t="inlineStr">
         <is>
-          <t>74469M</t>
+          <t>431616</t>
         </is>
       </c>
       <c r="I242" s="3" t="inlineStr">
@@ -38721,7 +38717,7 @@
       </c>
       <c r="H243" s="5" t="inlineStr">
         <is>
-          <t>74462M</t>
+          <t>431609</t>
         </is>
       </c>
       <c r="I243" s="5" t="inlineStr">
@@ -38764,7 +38760,7 @@
       </c>
       <c r="H244" s="3" t="inlineStr">
         <is>
-          <t>74413M</t>
+          <t>431560</t>
         </is>
       </c>
       <c r="I244" s="3" t="inlineStr">
@@ -38807,7 +38803,7 @@
       </c>
       <c r="H245" s="5" t="inlineStr">
         <is>
-          <t>80610M</t>
+          <t>437627</t>
         </is>
       </c>
       <c r="I245" s="5" t="inlineStr">
@@ -38850,7 +38846,7 @@
       </c>
       <c r="H246" s="3" t="inlineStr">
         <is>
-          <t>74456M</t>
+          <t>431603</t>
         </is>
       </c>
       <c r="I246" s="3" t="inlineStr">
@@ -38893,7 +38889,7 @@
       </c>
       <c r="H247" s="5" t="inlineStr">
         <is>
-          <t>74443M</t>
+          <t>431590</t>
         </is>
       </c>
       <c r="I247" s="5" t="inlineStr">
@@ -38936,7 +38932,7 @@
       </c>
       <c r="H248" s="3" t="inlineStr">
         <is>
-          <t>74461M</t>
+          <t>431608</t>
         </is>
       </c>
       <c r="I248" s="3" t="inlineStr">
@@ -38979,7 +38975,7 @@
       </c>
       <c r="H249" s="5" t="inlineStr">
         <is>
-          <t>74480M</t>
+          <t>431627</t>
         </is>
       </c>
       <c r="I249" s="5" t="inlineStr">
@@ -39022,7 +39018,7 @@
       </c>
       <c r="H250" s="3" t="inlineStr">
         <is>
-          <t>74438M</t>
+          <t>431584</t>
         </is>
       </c>
       <c r="I250" s="3" t="inlineStr">
@@ -39065,7 +39061,7 @@
       </c>
       <c r="H251" s="5" t="inlineStr">
         <is>
-          <t>74460M</t>
+          <t>431607</t>
         </is>
       </c>
       <c r="I251" s="5" t="inlineStr">
@@ -39108,7 +39104,7 @@
       </c>
       <c r="H252" s="3" t="inlineStr">
         <is>
-          <t>74476M</t>
+          <t>431622</t>
         </is>
       </c>
       <c r="I252" s="3" t="inlineStr">
@@ -39151,7 +39147,7 @@
       </c>
       <c r="H253" s="5" t="inlineStr">
         <is>
-          <t>74481M</t>
+          <t>431628</t>
         </is>
       </c>
       <c r="I253" s="5" t="inlineStr">
@@ -39194,7 +39190,7 @@
       </c>
       <c r="H254" s="3" t="inlineStr">
         <is>
-          <t>74429M</t>
+          <t>431576</t>
         </is>
       </c>
       <c r="I254" s="3" t="inlineStr">
@@ -39237,7 +39233,7 @@
       </c>
       <c r="H255" s="5" t="inlineStr">
         <is>
-          <t>74472M</t>
+          <t>431619</t>
         </is>
       </c>
       <c r="I255" s="5" t="inlineStr">
@@ -39280,7 +39276,7 @@
       </c>
       <c r="H256" s="3" t="inlineStr">
         <is>
-          <t>87917M</t>
+          <t>444922</t>
         </is>
       </c>
       <c r="I256" s="3" t="inlineStr">
@@ -39323,7 +39319,7 @@
       </c>
       <c r="H257" s="5" t="inlineStr">
         <is>
-          <t>74454M</t>
+          <t>431600</t>
         </is>
       </c>
       <c r="I257" s="5" t="inlineStr">
@@ -39366,7 +39362,7 @@
       </c>
       <c r="H258" s="3" t="inlineStr">
         <is>
-          <t>74428M</t>
+          <t>431574</t>
         </is>
       </c>
       <c r="I258" s="3" t="inlineStr">
@@ -39409,7 +39405,7 @@
       </c>
       <c r="H259" s="5" t="inlineStr">
         <is>
-          <t>74459M</t>
+          <t>431606</t>
         </is>
       </c>
       <c r="I259" s="5" t="inlineStr">
@@ -39452,7 +39448,7 @@
       </c>
       <c r="H260" s="3" t="inlineStr">
         <is>
-          <t>74486M</t>
+          <t>431633</t>
         </is>
       </c>
       <c r="I260" s="3" t="inlineStr">
@@ -39495,7 +39491,7 @@
       </c>
       <c r="H261" s="5" t="inlineStr">
         <is>
-          <t>74444M</t>
+          <t>431591</t>
         </is>
       </c>
       <c r="I261" s="5" t="inlineStr">
@@ -39538,7 +39534,7 @@
       </c>
       <c r="H262" s="3" t="inlineStr">
         <is>
-          <t>74470M</t>
+          <t>431617</t>
         </is>
       </c>
       <c r="I262" s="3" t="inlineStr">
@@ -39581,7 +39577,7 @@
       </c>
       <c r="H263" s="5" t="inlineStr">
         <is>
-          <t>74417M</t>
+          <t>431565</t>
         </is>
       </c>
       <c r="I263" s="5" t="inlineStr">
@@ -39624,7 +39620,7 @@
       </c>
       <c r="H264" s="3" t="inlineStr">
         <is>
-          <t>74440M</t>
+          <t>431586</t>
         </is>
       </c>
       <c r="I264" s="3" t="inlineStr">
@@ -39667,7 +39663,7 @@
       </c>
       <c r="H265" s="5" t="inlineStr">
         <is>
-          <t>74466M</t>
+          <t>431613</t>
         </is>
       </c>
       <c r="I265" s="5" t="inlineStr">
@@ -39710,7 +39706,7 @@
       </c>
       <c r="H266" s="3" t="inlineStr">
         <is>
-          <t>74467M</t>
+          <t>431614</t>
         </is>
       </c>
       <c r="I266" s="3" t="inlineStr">
@@ -39753,7 +39749,7 @@
       </c>
       <c r="H267" s="5" t="inlineStr">
         <is>
-          <t>74477M</t>
+          <t>431625</t>
         </is>
       </c>
       <c r="I267" s="5" t="inlineStr">
@@ -39796,7 +39792,7 @@
       </c>
       <c r="H268" s="3" t="inlineStr">
         <is>
-          <t>71092M</t>
+          <t>428238</t>
         </is>
       </c>
       <c r="I268" s="3" t="inlineStr">
@@ -39839,7 +39835,7 @@
       </c>
       <c r="H269" s="5" t="inlineStr">
         <is>
-          <t>71094M</t>
+          <t>428242</t>
         </is>
       </c>
       <c r="I269" s="5" t="inlineStr">
@@ -39882,7 +39878,7 @@
       </c>
       <c r="H270" s="3" t="inlineStr">
         <is>
-          <t>71142M</t>
+          <t>428290</t>
         </is>
       </c>
       <c r="I270" s="3" t="inlineStr">
@@ -39925,7 +39921,7 @@
       </c>
       <c r="H271" s="5" t="inlineStr">
         <is>
-          <t>71080M</t>
+          <t>428227</t>
         </is>
       </c>
       <c r="I271" s="5" t="inlineStr">
@@ -39968,7 +39964,7 @@
       </c>
       <c r="H272" s="3" t="inlineStr">
         <is>
-          <t>71141M</t>
+          <t>428288</t>
         </is>
       </c>
       <c r="I272" s="3" t="inlineStr">
@@ -40011,7 +40007,7 @@
       </c>
       <c r="H273" s="5" t="inlineStr">
         <is>
-          <t>71119M</t>
+          <t>428267</t>
         </is>
       </c>
       <c r="I273" s="5" t="inlineStr">
@@ -40054,7 +40050,7 @@
       </c>
       <c r="H274" s="3" t="inlineStr">
         <is>
-          <t>71041M</t>
+          <t>428187</t>
         </is>
       </c>
       <c r="I274" s="3" t="inlineStr">
@@ -40097,7 +40093,7 @@
       </c>
       <c r="H275" s="5" t="inlineStr">
         <is>
-          <t>71049M</t>
+          <t>428197</t>
         </is>
       </c>
       <c r="I275" s="5" t="inlineStr">
@@ -40140,7 +40136,7 @@
       </c>
       <c r="H276" s="3" t="inlineStr">
         <is>
-          <t>71043M</t>
+          <t>428190</t>
         </is>
       </c>
       <c r="I276" s="3" t="inlineStr">
@@ -40183,7 +40179,7 @@
       </c>
       <c r="H277" s="5" t="inlineStr">
         <is>
-          <t>71093M</t>
+          <t>428241</t>
         </is>
       </c>
       <c r="I277" s="5" t="inlineStr">
@@ -40226,7 +40222,7 @@
       </c>
       <c r="H278" s="7" t="inlineStr">
         <is>
-          <t>71069M</t>
+          <t>428215</t>
         </is>
       </c>
       <c r="I278" s="7" t="inlineStr">
@@ -40269,7 +40265,7 @@
       </c>
       <c r="H279" s="5" t="inlineStr">
         <is>
-          <t>71071M</t>
+          <t>428219</t>
         </is>
       </c>
       <c r="I279" s="5" t="inlineStr">
@@ -40312,7 +40308,7 @@
       </c>
       <c r="H280" s="3" t="inlineStr">
         <is>
-          <t>77796M</t>
+          <t>434878</t>
         </is>
       </c>
       <c r="I280" s="3" t="inlineStr">
@@ -40355,7 +40351,7 @@
       </c>
       <c r="H281" s="5" t="inlineStr">
         <is>
-          <t>71047M</t>
+          <t>428194</t>
         </is>
       </c>
       <c r="I281" s="5" t="inlineStr">
@@ -40398,7 +40394,7 @@
       </c>
       <c r="H282" s="3" t="inlineStr">
         <is>
-          <t>78223M</t>
+          <t>435279</t>
         </is>
       </c>
       <c r="I282" s="3" t="inlineStr">
@@ -40441,7 +40437,7 @@
       </c>
       <c r="H283" s="5" t="inlineStr">
         <is>
-          <t>71074M</t>
+          <t>428222</t>
         </is>
       </c>
       <c r="I283" s="5" t="inlineStr">
@@ -40484,7 +40480,7 @@
       </c>
       <c r="H284" s="3" t="inlineStr">
         <is>
-          <t>71096M</t>
+          <t>428243</t>
         </is>
       </c>
       <c r="I284" s="3" t="inlineStr">
@@ -40527,7 +40523,7 @@
       </c>
       <c r="H285" s="5" t="inlineStr">
         <is>
-          <t>71116M</t>
+          <t>428263</t>
         </is>
       </c>
       <c r="I285" s="5" t="inlineStr">
@@ -40570,7 +40566,7 @@
       </c>
       <c r="H286" s="3" t="inlineStr">
         <is>
-          <t>71038M</t>
+          <t>428184</t>
         </is>
       </c>
       <c r="I286" s="3" t="inlineStr">
@@ -40613,7 +40609,7 @@
       </c>
       <c r="H287" s="5" t="inlineStr">
         <is>
-          <t>77805M</t>
+          <t>434887</t>
         </is>
       </c>
       <c r="I287" s="5" t="inlineStr">
@@ -40656,7 +40652,7 @@
       </c>
       <c r="H288" s="3" t="inlineStr">
         <is>
-          <t>71086M</t>
+          <t>428233</t>
         </is>
       </c>
       <c r="I288" s="3" t="inlineStr">
@@ -40699,7 +40695,7 @@
       </c>
       <c r="H289" s="5" t="inlineStr">
         <is>
-          <t>71179M</t>
+          <t>428327</t>
         </is>
       </c>
       <c r="I289" s="5" t="inlineStr">
@@ -40742,7 +40738,7 @@
       </c>
       <c r="H290" s="3" t="inlineStr">
         <is>
-          <t>88057M</t>
+          <t>445062</t>
         </is>
       </c>
       <c r="I290" s="3" t="inlineStr">
@@ -40785,7 +40781,7 @@
       </c>
       <c r="H291" s="5" t="inlineStr">
         <is>
-          <t>71059M</t>
+          <t>428206</t>
         </is>
       </c>
       <c r="I291" s="5" t="inlineStr">
@@ -40828,7 +40824,7 @@
       </c>
       <c r="H292" s="3" t="inlineStr">
         <is>
-          <t>71114M</t>
+          <t>428262</t>
         </is>
       </c>
       <c r="I292" s="3" t="inlineStr">
@@ -40871,7 +40867,7 @@
       </c>
       <c r="H293" s="5" t="inlineStr">
         <is>
-          <t>71098M</t>
+          <t>428246</t>
         </is>
       </c>
       <c r="I293" s="5" t="inlineStr">
@@ -40914,7 +40910,7 @@
       </c>
       <c r="H294" s="3" t="inlineStr">
         <is>
-          <t>71078M</t>
+          <t>428226</t>
         </is>
       </c>
       <c r="I294" s="3" t="inlineStr">
@@ -40957,7 +40953,7 @@
       </c>
       <c r="H295" s="5" t="inlineStr">
         <is>
-          <t>71075M</t>
+          <t>428223</t>
         </is>
       </c>
       <c r="I295" s="5" t="inlineStr">
@@ -41000,7 +40996,7 @@
       </c>
       <c r="H296" s="3" t="inlineStr">
         <is>
-          <t>71060M</t>
+          <t>428208</t>
         </is>
       </c>
       <c r="I296" s="3" t="inlineStr">
@@ -41043,7 +41039,7 @@
       </c>
       <c r="H297" s="5" t="inlineStr">
         <is>
-          <t>71048M</t>
+          <t>428196</t>
         </is>
       </c>
       <c r="I297" s="5" t="inlineStr">
@@ -41086,7 +41082,7 @@
       </c>
       <c r="H298" s="3" t="inlineStr">
         <is>
-          <t>71089M</t>
+          <t>428237</t>
         </is>
       </c>
       <c r="I298" s="3" t="inlineStr">
@@ -41129,7 +41125,7 @@
       </c>
       <c r="H299" s="5" t="inlineStr">
         <is>
-          <t>71111M</t>
+          <t>428259</t>
         </is>
       </c>
       <c r="I299" s="5" t="inlineStr">
@@ -41172,7 +41168,7 @@
       </c>
       <c r="H300" s="3" t="inlineStr">
         <is>
-          <t>71088M</t>
+          <t>428236</t>
         </is>
       </c>
       <c r="I300" s="3" t="inlineStr">
@@ -41215,7 +41211,7 @@
       </c>
       <c r="H301" s="5" t="inlineStr">
         <is>
-          <t>71055M</t>
+          <t>428201</t>
         </is>
       </c>
       <c r="I301" s="5" t="inlineStr">
@@ -41258,7 +41254,7 @@
       </c>
       <c r="H302" s="3" t="inlineStr">
         <is>
-          <t>71083M</t>
+          <t>428231</t>
         </is>
       </c>
       <c r="I302" s="3" t="inlineStr">
@@ -41301,7 +41297,7 @@
       </c>
       <c r="H303" s="5" t="inlineStr">
         <is>
-          <t>88359M</t>
+          <t>445360</t>
         </is>
       </c>
       <c r="I303" s="5" t="inlineStr">
@@ -41344,7 +41340,7 @@
       </c>
       <c r="H304" s="3" t="inlineStr">
         <is>
-          <t>71045M</t>
+          <t>428192</t>
         </is>
       </c>
       <c r="I304" s="3" t="inlineStr">
@@ -41387,7 +41383,7 @@
       </c>
       <c r="H305" s="5" t="inlineStr">
         <is>
-          <t>71101M</t>
+          <t>428248</t>
         </is>
       </c>
       <c r="I305" s="5" t="inlineStr">
@@ -41430,7 +41426,7 @@
       </c>
       <c r="H306" s="3" t="inlineStr">
         <is>
-          <t>71062M</t>
+          <t>428210</t>
         </is>
       </c>
       <c r="I306" s="3" t="inlineStr">
@@ -41473,7 +41469,7 @@
       </c>
       <c r="H307" s="7" t="inlineStr">
         <is>
-          <t>71057M</t>
+          <t>428205</t>
         </is>
       </c>
       <c r="I307" s="7" t="inlineStr">
@@ -41516,7 +41512,7 @@
       </c>
       <c r="H308" s="3" t="inlineStr">
         <is>
-          <t>88060M</t>
+          <t>445065</t>
         </is>
       </c>
       <c r="I308" s="3" t="inlineStr">
@@ -41559,7 +41555,7 @@
       </c>
       <c r="H309" s="7" t="inlineStr">
         <is>
-          <t>71077M</t>
+          <t>428224</t>
         </is>
       </c>
       <c r="I309" s="7" t="inlineStr">
@@ -41602,7 +41598,7 @@
       </c>
       <c r="H310" s="3" t="inlineStr">
         <is>
-          <t>71061M</t>
+          <t>428209</t>
         </is>
       </c>
       <c r="I310" s="3" t="inlineStr">
@@ -41645,7 +41641,7 @@
       </c>
       <c r="H311" s="5" t="inlineStr">
         <is>
-          <t>71035M</t>
+          <t>428182</t>
         </is>
       </c>
       <c r="I311" s="5" t="inlineStr">
@@ -41688,7 +41684,7 @@
       </c>
       <c r="H312" s="3" t="inlineStr">
         <is>
-          <t>71066M</t>
+          <t>428214</t>
         </is>
       </c>
       <c r="I312" s="3" t="inlineStr">
@@ -41731,7 +41727,7 @@
       </c>
       <c r="H313" s="5" t="inlineStr">
         <is>
-          <t>88059M</t>
+          <t>445064</t>
         </is>
       </c>
       <c r="I313" s="5" t="inlineStr">
@@ -41774,7 +41770,7 @@
       </c>
       <c r="H314" s="3" t="inlineStr">
         <is>
-          <t>71132M</t>
+          <t>428280</t>
         </is>
       </c>
       <c r="I314" s="3" t="inlineStr">
@@ -41817,7 +41813,7 @@
       </c>
       <c r="H315" s="5" t="inlineStr">
         <is>
-          <t>71039M</t>
+          <t>428188</t>
         </is>
       </c>
       <c r="I315" s="5" t="inlineStr">
@@ -41860,7 +41856,7 @@
       </c>
       <c r="H316" s="3" t="inlineStr">
         <is>
-          <t>71118M</t>
+          <t>428266</t>
         </is>
       </c>
       <c r="I316" s="3" t="inlineStr">
@@ -41903,7 +41899,7 @@
       </c>
       <c r="H317" s="7" t="inlineStr">
         <is>
-          <t>71117M</t>
+          <t>428265</t>
         </is>
       </c>
       <c r="I317" s="7" t="inlineStr">
@@ -41946,7 +41942,7 @@
       </c>
       <c r="H318" s="7" t="inlineStr">
         <is>
-          <t>71065M</t>
+          <t>428213</t>
         </is>
       </c>
       <c r="I318" s="7" t="inlineStr">
@@ -41989,7 +41985,7 @@
       </c>
       <c r="H319" s="5" t="inlineStr">
         <is>
-          <t>71073M</t>
+          <t>428221</t>
         </is>
       </c>
       <c r="I319" s="5" t="inlineStr">
@@ -42032,7 +42028,7 @@
       </c>
       <c r="H320" s="3" t="inlineStr">
         <is>
-          <t>71051M</t>
+          <t>428198</t>
         </is>
       </c>
       <c r="I320" s="3" t="inlineStr">
@@ -42075,7 +42071,7 @@
       </c>
       <c r="H321" s="5" t="inlineStr">
         <is>
-          <t>71108M</t>
+          <t>428256</t>
         </is>
       </c>
       <c r="I321" s="5" t="inlineStr">
@@ -42118,7 +42114,7 @@
       </c>
       <c r="H322" s="3" t="inlineStr">
         <is>
-          <t>71102M</t>
+          <t>428250</t>
         </is>
       </c>
       <c r="I322" s="3" t="inlineStr">
@@ -42161,7 +42157,7 @@
       </c>
       <c r="H323" s="5" t="inlineStr">
         <is>
-          <t>79053M</t>
+          <t>436086</t>
         </is>
       </c>
       <c r="I323" s="5" t="inlineStr">
@@ -42204,7 +42200,7 @@
       </c>
       <c r="H324" s="3" t="inlineStr">
         <is>
-          <t>71107M</t>
+          <t>428255</t>
         </is>
       </c>
       <c r="I324" s="3" t="inlineStr">
@@ -42247,7 +42243,7 @@
       </c>
       <c r="H325" s="5" t="inlineStr">
         <is>
-          <t>71123M</t>
+          <t>428271</t>
         </is>
       </c>
       <c r="I325" s="5" t="inlineStr">
@@ -42290,7 +42286,7 @@
       </c>
       <c r="H326" s="3" t="inlineStr">
         <is>
-          <t>71124M</t>
+          <t>428272</t>
         </is>
       </c>
       <c r="I326" s="3" t="inlineStr">
@@ -42333,7 +42329,7 @@
       </c>
       <c r="H327" s="5" t="inlineStr">
         <is>
-          <t>71129M</t>
+          <t>428277</t>
         </is>
       </c>
       <c r="I327" s="5" t="inlineStr">
@@ -42376,7 +42372,7 @@
       </c>
       <c r="H328" s="3" t="inlineStr">
         <is>
-          <t>71081M</t>
+          <t>428230</t>
         </is>
       </c>
       <c r="I328" s="3" t="inlineStr">
@@ -42419,7 +42415,7 @@
       </c>
       <c r="H329" s="5" t="inlineStr">
         <is>
-          <t>71138M</t>
+          <t>428286</t>
         </is>
       </c>
       <c r="I329" s="5" t="inlineStr">
@@ -42462,7 +42458,7 @@
       </c>
       <c r="H330" s="3" t="inlineStr">
         <is>
-          <t>71181M</t>
+          <t>428329</t>
         </is>
       </c>
       <c r="I330" s="3" t="inlineStr">
@@ -42505,7 +42501,7 @@
       </c>
       <c r="H331" s="5" t="inlineStr">
         <is>
-          <t>71104M</t>
+          <t>428252</t>
         </is>
       </c>
       <c r="I331" s="5" t="inlineStr">
@@ -42548,7 +42544,7 @@
       </c>
       <c r="H332" s="3" t="inlineStr">
         <is>
-          <t>71110M</t>
+          <t>428257</t>
         </is>
       </c>
       <c r="I332" s="3" t="inlineStr">
@@ -42591,7 +42587,7 @@
       </c>
       <c r="H333" s="5" t="inlineStr">
         <is>
-          <t>71064M</t>
+          <t>428211</t>
         </is>
       </c>
       <c r="I333" s="5" t="inlineStr">
@@ -42634,7 +42630,7 @@
       </c>
       <c r="H334" s="3" t="inlineStr">
         <is>
-          <t>71113M</t>
+          <t>428260</t>
         </is>
       </c>
       <c r="I334" s="3" t="inlineStr">
@@ -42677,7 +42673,7 @@
       </c>
       <c r="H335" s="5" t="inlineStr">
         <is>
-          <t>78239M</t>
+          <t>435295</t>
         </is>
       </c>
       <c r="I335" s="5" t="inlineStr">
@@ -42720,7 +42716,7 @@
       </c>
       <c r="H336" s="3" t="inlineStr">
         <is>
-          <t>86589M</t>
+          <t>443596</t>
         </is>
       </c>
       <c r="I336" s="3" t="inlineStr">
@@ -42763,7 +42759,7 @@
       </c>
       <c r="H337" s="5" t="inlineStr">
         <is>
-          <t>71125M</t>
+          <t>428273</t>
         </is>
       </c>
       <c r="I337" s="5" t="inlineStr">
@@ -42806,7 +42802,7 @@
       </c>
       <c r="H338" s="3" t="inlineStr">
         <is>
-          <t>71135M</t>
+          <t>428283</t>
         </is>
       </c>
       <c r="I338" s="3" t="inlineStr">
@@ -42849,7 +42845,7 @@
       </c>
       <c r="H339" s="5" t="inlineStr">
         <is>
-          <t>71139M</t>
+          <t>428287</t>
         </is>
       </c>
       <c r="I339" s="5" t="inlineStr">
@@ -42892,7 +42888,7 @@
       </c>
       <c r="H340" s="3" t="inlineStr">
         <is>
-          <t>71128M</t>
+          <t>428276</t>
         </is>
       </c>
       <c r="I340" s="3" t="inlineStr">
@@ -42935,7 +42931,7 @@
       </c>
       <c r="H341" s="5" t="inlineStr">
         <is>
-          <t>71121M</t>
+          <t>428269</t>
         </is>
       </c>
       <c r="I341" s="5" t="inlineStr">
@@ -42978,7 +42974,7 @@
       </c>
       <c r="H342" s="7" t="inlineStr">
         <is>
-          <t>71052M</t>
+          <t>428200</t>
         </is>
       </c>
       <c r="I342" s="7" t="inlineStr">
@@ -43021,7 +43017,7 @@
       </c>
       <c r="H343" s="5" t="inlineStr">
         <is>
-          <t>71130M</t>
+          <t>428278</t>
         </is>
       </c>
       <c r="I343" s="5" t="inlineStr">
@@ -43064,7 +43060,7 @@
       </c>
       <c r="H344" s="3" t="inlineStr">
         <is>
-          <t>87915M</t>
+          <t>444920</t>
         </is>
       </c>
       <c r="I344" s="3" t="inlineStr">
@@ -43107,7 +43103,7 @@
       </c>
       <c r="H345" s="5" t="inlineStr">
         <is>
-          <t>88039M</t>
+          <t>445044</t>
         </is>
       </c>
       <c r="I345" s="5" t="inlineStr">
@@ -43150,7 +43146,7 @@
       </c>
       <c r="H346" s="3" t="inlineStr">
         <is>
-          <t>71137M</t>
+          <t>428285</t>
         </is>
       </c>
       <c r="I346" s="3" t="inlineStr">
@@ -43193,7 +43189,7 @@
       </c>
       <c r="H347" s="5" t="inlineStr">
         <is>
-          <t>71134M</t>
+          <t>428282</t>
         </is>
       </c>
       <c r="I347" s="5" t="inlineStr">
@@ -43236,7 +43232,7 @@
       </c>
       <c r="H348" s="3" t="inlineStr">
         <is>
-          <t>71097M</t>
+          <t>428245</t>
         </is>
       </c>
       <c r="I348" s="3" t="inlineStr">
@@ -43279,7 +43275,7 @@
       </c>
       <c r="H349" s="5" t="inlineStr">
         <is>
-          <t>71106M</t>
+          <t>428254</t>
         </is>
       </c>
       <c r="I349" s="5" t="inlineStr">
@@ -43322,7 +43318,7 @@
       </c>
       <c r="H350" s="3" t="inlineStr">
         <is>
-          <t>71056M</t>
+          <t>428204</t>
         </is>
       </c>
       <c r="I350" s="3" t="inlineStr">
@@ -43365,7 +43361,7 @@
       </c>
       <c r="H351" s="5" t="inlineStr">
         <is>
-          <t>71143M</t>
+          <t>428291</t>
         </is>
       </c>
       <c r="I351" s="5" t="inlineStr">
@@ -43408,7 +43404,7 @@
       </c>
       <c r="H352" s="3" t="inlineStr">
         <is>
-          <t>71120M</t>
+          <t>428268</t>
         </is>
       </c>
       <c r="I352" s="3" t="inlineStr">
@@ -43451,7 +43447,7 @@
       </c>
       <c r="H353" s="5" t="inlineStr">
         <is>
-          <t>71131M</t>
+          <t>428279</t>
         </is>
       </c>
       <c r="I353" s="5" t="inlineStr">
@@ -43494,7 +43490,7 @@
       </c>
       <c r="H354" s="3" t="inlineStr">
         <is>
-          <t>71122M</t>
+          <t>428270</t>
         </is>
       </c>
       <c r="I354" s="3" t="inlineStr">
@@ -43537,7 +43533,7 @@
       </c>
       <c r="H355" s="5" t="inlineStr">
         <is>
-          <t>71099M</t>
+          <t>428247</t>
         </is>
       </c>
       <c r="I355" s="5" t="inlineStr">
@@ -43580,7 +43576,7 @@
       </c>
       <c r="H356" s="7" t="inlineStr">
         <is>
-          <t>71000M</t>
+          <t>428148</t>
         </is>
       </c>
       <c r="I356" s="7" t="inlineStr">
@@ -43623,7 +43619,7 @@
       </c>
       <c r="H357" s="5" t="inlineStr">
         <is>
-          <t>77803M</t>
+          <t>434885</t>
         </is>
       </c>
       <c r="I357" s="5" t="inlineStr">
@@ -43666,7 +43662,7 @@
       </c>
       <c r="H358" s="3" t="inlineStr">
         <is>
-          <t>71001M</t>
+          <t>428149</t>
         </is>
       </c>
       <c r="I358" s="3" t="inlineStr">
@@ -43709,7 +43705,7 @@
       </c>
       <c r="H359" s="5" t="inlineStr">
         <is>
-          <t>71027M</t>
+          <t>428175</t>
         </is>
       </c>
       <c r="I359" s="5" t="inlineStr">
@@ -43752,7 +43748,7 @@
       </c>
       <c r="H360" s="3" t="inlineStr">
         <is>
-          <t>71726M</t>
+          <t>428874</t>
         </is>
       </c>
       <c r="I360" s="3" t="inlineStr">
@@ -43795,7 +43791,7 @@
       </c>
       <c r="H361" s="5" t="inlineStr">
         <is>
-          <t>71010M</t>
+          <t>428158</t>
         </is>
       </c>
       <c r="I361" s="5" t="inlineStr">
@@ -43838,7 +43834,7 @@
       </c>
       <c r="H362" s="3" t="inlineStr">
         <is>
-          <t>71011M</t>
+          <t>428159</t>
         </is>
       </c>
       <c r="I362" s="3" t="inlineStr">
@@ -43881,7 +43877,7 @@
       </c>
       <c r="H363" s="5" t="inlineStr">
         <is>
-          <t>71018M</t>
+          <t>428165</t>
         </is>
       </c>
       <c r="I363" s="5" t="inlineStr">
@@ -43924,7 +43920,7 @@
       </c>
       <c r="H364" s="3" t="inlineStr">
         <is>
-          <t>71722M</t>
+          <t>428870</t>
         </is>
       </c>
       <c r="I364" s="3" t="inlineStr">
@@ -43967,7 +43963,7 @@
       </c>
       <c r="H365" s="5" t="inlineStr">
         <is>
-          <t>71718M</t>
+          <t>428866</t>
         </is>
       </c>
       <c r="I365" s="5" t="inlineStr">
@@ -44010,7 +44006,7 @@
       </c>
       <c r="H366" s="3" t="inlineStr">
         <is>
-          <t>71025M</t>
+          <t>428173</t>
         </is>
       </c>
       <c r="I366" s="3" t="inlineStr">
@@ -44053,7 +44049,7 @@
       </c>
       <c r="H367" s="5" t="inlineStr">
         <is>
-          <t>71013M</t>
+          <t>428161</t>
         </is>
       </c>
       <c r="I367" s="5" t="inlineStr">
@@ -44096,7 +44092,7 @@
       </c>
       <c r="H368" s="3" t="inlineStr">
         <is>
-          <t>71009M</t>
+          <t>428157</t>
         </is>
       </c>
       <c r="I368" s="3" t="inlineStr">
@@ -44139,7 +44135,7 @@
       </c>
       <c r="H369" s="5" t="inlineStr">
         <is>
-          <t>77802M</t>
+          <t>434884</t>
         </is>
       </c>
       <c r="I369" s="5" t="inlineStr">
@@ -44182,7 +44178,7 @@
       </c>
       <c r="H370" s="3" t="inlineStr">
         <is>
-          <t>70989M</t>
+          <t>428137</t>
         </is>
       </c>
       <c r="I370" s="3" t="inlineStr">
@@ -44225,7 +44221,7 @@
       </c>
       <c r="H371" s="5" t="inlineStr">
         <is>
-          <t>71028M</t>
+          <t>428176</t>
         </is>
       </c>
       <c r="I371" s="5" t="inlineStr">
@@ -44268,7 +44264,7 @@
       </c>
       <c r="H372" s="3" t="inlineStr">
         <is>
-          <t>70986M</t>
+          <t>428134</t>
         </is>
       </c>
       <c r="I372" s="3" t="inlineStr">
@@ -44311,7 +44307,7 @@
       </c>
       <c r="H373" s="5" t="inlineStr">
         <is>
-          <t>71720M</t>
+          <t>428868</t>
         </is>
       </c>
       <c r="I373" s="5" t="inlineStr">
@@ -44354,7 +44350,7 @@
       </c>
       <c r="H374" s="3" t="inlineStr">
         <is>
-          <t>77801M</t>
+          <t>434883</t>
         </is>
       </c>
       <c r="I374" s="3" t="inlineStr">
@@ -44397,7 +44393,7 @@
       </c>
       <c r="H375" s="5" t="inlineStr">
         <is>
-          <t>71724M</t>
+          <t>428872</t>
         </is>
       </c>
       <c r="I375" s="5" t="inlineStr">
@@ -44440,7 +44436,7 @@
       </c>
       <c r="H376" s="3" t="inlineStr">
         <is>
-          <t>77799M</t>
+          <t>434881</t>
         </is>
       </c>
       <c r="I376" s="3" t="inlineStr">
@@ -44483,7 +44479,7 @@
       </c>
       <c r="H377" s="5" t="inlineStr">
         <is>
-          <t>71022M</t>
+          <t>428170</t>
         </is>
       </c>
       <c r="I377" s="5" t="inlineStr">
@@ -44526,7 +44522,7 @@
       </c>
       <c r="H378" s="3" t="inlineStr">
         <is>
-          <t>71005M</t>
+          <t>428153</t>
         </is>
       </c>
       <c r="I378" s="3" t="inlineStr">
@@ -44569,7 +44565,7 @@
       </c>
       <c r="H379" s="5" t="inlineStr">
         <is>
-          <t>70980M</t>
+          <t>428128</t>
         </is>
       </c>
       <c r="I379" s="5" t="inlineStr">
@@ -44612,7 +44608,7 @@
       </c>
       <c r="H380" s="3" t="inlineStr">
         <is>
-          <t>70995M</t>
+          <t>428143</t>
         </is>
       </c>
       <c r="I380" s="3" t="inlineStr">
@@ -44655,7 +44651,7 @@
       </c>
       <c r="H381" s="5" t="inlineStr">
         <is>
-          <t>71008M</t>
+          <t>428156</t>
         </is>
       </c>
       <c r="I381" s="5" t="inlineStr">
@@ -44698,7 +44694,7 @@
       </c>
       <c r="H382" s="3" t="inlineStr">
         <is>
-          <t>77797M</t>
+          <t>434879</t>
         </is>
       </c>
       <c r="I382" s="3" t="inlineStr">
@@ -44741,7 +44737,7 @@
       </c>
       <c r="H383" s="5" t="inlineStr">
         <is>
-          <t>71725M</t>
+          <t>428873</t>
         </is>
       </c>
       <c r="I383" s="5" t="inlineStr">
@@ -44784,7 +44780,7 @@
       </c>
       <c r="H384" s="7" t="inlineStr">
         <is>
-          <t>70994M</t>
+          <t>428142</t>
         </is>
       </c>
       <c r="I384" s="7" t="inlineStr">
@@ -44827,7 +44823,7 @@
       </c>
       <c r="H385" s="5" t="inlineStr">
         <is>
-          <t>71006M</t>
+          <t>428154</t>
         </is>
       </c>
       <c r="I385" s="5" t="inlineStr">
@@ -44870,7 +44866,7 @@
       </c>
       <c r="H386" s="3" t="inlineStr">
         <is>
-          <t>70982M</t>
+          <t>428130</t>
         </is>
       </c>
       <c r="I386" s="3" t="inlineStr">
@@ -44913,7 +44909,7 @@
       </c>
       <c r="H387" s="5" t="inlineStr">
         <is>
-          <t>70999M</t>
+          <t>428147</t>
         </is>
       </c>
       <c r="I387" s="5" t="inlineStr">
@@ -44956,7 +44952,7 @@
       </c>
       <c r="H388" s="3" t="inlineStr">
         <is>
-          <t>71026M</t>
+          <t>428174</t>
         </is>
       </c>
       <c r="I388" s="3" t="inlineStr">
@@ -44999,7 +44995,7 @@
       </c>
       <c r="H389" s="5" t="inlineStr">
         <is>
-          <t>77804M</t>
+          <t>434886</t>
         </is>
       </c>
       <c r="I389" s="5" t="inlineStr">
@@ -45042,7 +45038,7 @@
       </c>
       <c r="H390" s="3" t="inlineStr">
         <is>
-          <t>71015M</t>
+          <t>428162</t>
         </is>
       </c>
       <c r="I390" s="3" t="inlineStr">
@@ -45085,7 +45081,7 @@
       </c>
       <c r="H391" s="5" t="inlineStr">
         <is>
-          <t>71021M</t>
+          <t>428169</t>
         </is>
       </c>
       <c r="I391" s="5" t="inlineStr">
@@ -45128,7 +45124,7 @@
       </c>
       <c r="H392" s="3" t="inlineStr">
         <is>
-          <t>71023M</t>
+          <t>428171</t>
         </is>
       </c>
       <c r="I392" s="3" t="inlineStr">
@@ -45171,7 +45167,7 @@
       </c>
       <c r="H393" s="5" t="inlineStr">
         <is>
-          <t>71016M</t>
+          <t>428164</t>
         </is>
       </c>
       <c r="I393" s="5" t="inlineStr">
@@ -45214,7 +45210,7 @@
       </c>
       <c r="H394" s="3" t="inlineStr">
         <is>
-          <t>70997M</t>
+          <t>428145</t>
         </is>
       </c>
       <c r="I394" s="3" t="inlineStr">
@@ -45257,7 +45253,7 @@
       </c>
       <c r="H395" s="5" t="inlineStr">
         <is>
-          <t>71003M</t>
+          <t>428150</t>
         </is>
       </c>
       <c r="I395" s="5" t="inlineStr">
@@ -45300,7 +45296,7 @@
       </c>
       <c r="H396" s="3" t="inlineStr">
         <is>
-          <t>70983M</t>
+          <t>428131</t>
         </is>
       </c>
       <c r="I396" s="3" t="inlineStr">
@@ -45343,7 +45339,7 @@
       </c>
       <c r="H397" s="5" t="inlineStr">
         <is>
-          <t>71030M</t>
+          <t>428178</t>
         </is>
       </c>
       <c r="I397" s="5" t="inlineStr">
@@ -45386,7 +45382,7 @@
       </c>
       <c r="H398" s="3" t="inlineStr">
         <is>
-          <t>71029M</t>
+          <t>428177</t>
         </is>
       </c>
       <c r="I398" s="3" t="inlineStr">
@@ -45429,7 +45425,7 @@
       </c>
       <c r="H399" s="5" t="inlineStr">
         <is>
-          <t>86589M</t>
+          <t>443596</t>
         </is>
       </c>
       <c r="I399" s="5" t="inlineStr">
@@ -45472,7 +45468,7 @@
       </c>
       <c r="H400" s="3" t="inlineStr">
         <is>
-          <t>88037M</t>
+          <t>445043</t>
         </is>
       </c>
       <c r="I400" s="3" t="inlineStr">
@@ -45515,7 +45511,7 @@
       </c>
       <c r="H401" s="5" t="inlineStr">
         <is>
-          <t>70996M</t>
+          <t>428144</t>
         </is>
       </c>
       <c r="I401" s="5" t="inlineStr">
@@ -45558,7 +45554,7 @@
       </c>
       <c r="H402" s="3" t="inlineStr">
         <is>
-          <t>71012M</t>
+          <t>428160</t>
         </is>
       </c>
       <c r="I402" s="3" t="inlineStr">
@@ -45601,7 +45597,7 @@
       </c>
       <c r="H403" s="5" t="inlineStr">
         <is>
-          <t>71729M</t>
+          <t>428877</t>
         </is>
       </c>
       <c r="I403" s="5" t="inlineStr">
@@ -45644,7 +45640,7 @@
       </c>
       <c r="H404" s="3" t="inlineStr">
         <is>
-          <t>77798M</t>
+          <t>434880</t>
         </is>
       </c>
       <c r="I404" s="3" t="inlineStr">
@@ -45687,7 +45683,7 @@
       </c>
       <c r="H405" s="5" t="inlineStr">
         <is>
-          <t>70988M</t>
+          <t>428136</t>
         </is>
       </c>
       <c r="I405" s="5" t="inlineStr">
@@ -45730,7 +45726,7 @@
       </c>
       <c r="H406" s="3" t="inlineStr">
         <is>
-          <t>71007M</t>
+          <t>428155</t>
         </is>
       </c>
       <c r="I406" s="3" t="inlineStr">
@@ -45773,7 +45769,7 @@
       </c>
       <c r="H407" s="5" t="inlineStr">
         <is>
-          <t>71032M</t>
+          <t>428180</t>
         </is>
       </c>
       <c r="I407" s="5" t="inlineStr">
@@ -45816,7 +45812,7 @@
       </c>
       <c r="H408" s="3" t="inlineStr">
         <is>
-          <t>71727M</t>
+          <t>428875</t>
         </is>
       </c>
       <c r="I408" s="3" t="inlineStr">
@@ -45859,7 +45855,7 @@
       </c>
       <c r="H409" s="5" t="inlineStr">
         <is>
-          <t>71730M</t>
+          <t>428878</t>
         </is>
       </c>
       <c r="I409" s="5" t="inlineStr">
@@ -45902,7 +45898,7 @@
       </c>
       <c r="H410" s="3" t="inlineStr">
         <is>
-          <t>88039M</t>
+          <t>445044</t>
         </is>
       </c>
       <c r="I410" s="3" t="inlineStr">
@@ -45945,7 +45941,7 @@
       </c>
       <c r="H411" s="5" t="inlineStr">
         <is>
-          <t>71031M</t>
+          <t>428179</t>
         </is>
       </c>
       <c r="I411" s="5" t="inlineStr">
@@ -45988,7 +45984,7 @@
       </c>
       <c r="H412" s="3" t="inlineStr">
         <is>
-          <t>70981M</t>
+          <t>428129</t>
         </is>
       </c>
       <c r="I412" s="3" t="inlineStr">
@@ -46031,7 +46027,7 @@
       </c>
       <c r="H413" s="5" t="inlineStr">
         <is>
-          <t>70984M</t>
+          <t>428132</t>
         </is>
       </c>
       <c r="I413" s="5" t="inlineStr">
@@ -46074,7 +46070,7 @@
       </c>
       <c r="H414" s="3" t="inlineStr">
         <is>
-          <t>70991M</t>
+          <t>428139</t>
         </is>
       </c>
       <c r="I414" s="3" t="inlineStr">
@@ -46117,7 +46113,7 @@
       </c>
       <c r="H415" s="5" t="inlineStr">
         <is>
-          <t>70993M</t>
+          <t>428141</t>
         </is>
       </c>
       <c r="I415" s="5" t="inlineStr">
@@ -46160,7 +46156,7 @@
       </c>
       <c r="H416" s="3" t="inlineStr">
         <is>
-          <t>70985M</t>
+          <t>428133</t>
         </is>
       </c>
       <c r="I416" s="3" t="inlineStr">
@@ -46203,7 +46199,7 @@
       </c>
       <c r="H417" s="5" t="inlineStr">
         <is>
-          <t>70987M</t>
+          <t>428135</t>
         </is>
       </c>
       <c r="I417" s="5" t="inlineStr">
@@ -46246,7 +46242,7 @@
       </c>
       <c r="H418" s="3" t="inlineStr">
         <is>
-          <t>70990M</t>
+          <t>428138</t>
         </is>
       </c>
       <c r="I418" s="3" t="inlineStr">
@@ -46289,7 +46285,7 @@
       </c>
       <c r="H419" s="5" t="inlineStr">
         <is>
-          <t>88036M</t>
+          <t>445041</t>
         </is>
       </c>
       <c r="I419" s="5" t="inlineStr">
@@ -46332,7 +46328,7 @@
       </c>
       <c r="H420" s="3" t="inlineStr">
         <is>
-          <t>70992M</t>
+          <t>428140</t>
         </is>
       </c>
       <c r="I420" s="3" t="inlineStr">
@@ -46375,7 +46371,7 @@
       </c>
       <c r="H421" s="5" t="inlineStr">
         <is>
-          <t>70998M</t>
+          <t>428146</t>
         </is>
       </c>
       <c r="I421" s="5" t="inlineStr">
@@ -46418,7 +46414,7 @@
       </c>
       <c r="H422" s="3" t="inlineStr">
         <is>
-          <t>77800M</t>
+          <t>434882</t>
         </is>
       </c>
       <c r="I422" s="3" t="inlineStr">
@@ -46461,7 +46457,7 @@
       </c>
       <c r="H423" s="5" t="inlineStr">
         <is>
-          <t>71004M</t>
+          <t>428152</t>
         </is>
       </c>
       <c r="I423" s="5" t="inlineStr">
@@ -46504,7 +46500,7 @@
       </c>
       <c r="H424" s="3" t="inlineStr">
         <is>
-          <t>71019M</t>
+          <t>428167</t>
         </is>
       </c>
       <c r="I424" s="3" t="inlineStr">
@@ -46547,7 +46543,7 @@
       </c>
       <c r="H425" s="5" t="inlineStr">
         <is>
-          <t>71020M</t>
+          <t>428168</t>
         </is>
       </c>
       <c r="I425" s="5" t="inlineStr">
@@ -46590,7 +46586,7 @@
       </c>
       <c r="H426" s="3" t="inlineStr">
         <is>
-          <t>71024M</t>
+          <t>428172</t>
         </is>
       </c>
       <c r="I426" s="3" t="inlineStr">
@@ -46633,7 +46629,7 @@
       </c>
       <c r="H427" s="5" t="inlineStr">
         <is>
-          <t>71033M</t>
+          <t>428181</t>
         </is>
       </c>
       <c r="I427" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-05-31 20:44 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_31_05_2026.xlsx
+++ b/logs/Consolidado_31_05_2026.xlsx
@@ -14263,11 +14263,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>6661442</t>
-        </is>
-      </c>
+      <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
           <t>30%</t>
@@ -18656,7 +18652,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>6490926</t>
+        </is>
+      </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
           <t>28%</t>

</xml_diff>